<commit_message>
se implementa liquidacion consolidada
</commit_message>
<xml_diff>
--- a/plantillas_excel/PLANTILLA_POSTE_A_POSTE_AP.xlsx
+++ b/plantillas_excel/PLANTILLA_POSTE_A_POSTE_AP.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORMATO POSTE A POSTE AP" sheetId="1" state="visible" r:id="rId1"/>
@@ -1857,7 +1857,7 @@
   <sheetPr>
     <tabColor theme="5" tint="0.7999816888943144"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:AY40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
@@ -2661,7 +2661,7 @@
       <c r="AX11" s="232" t="n"/>
       <c r="AY11" s="233" t="n"/>
     </row>
-    <row r="12" ht="18" customHeight="1">
+    <row r="12" ht="58.5" customHeight="1">
       <c r="A12" s="234" t="n"/>
       <c r="B12" s="234" t="n"/>
       <c r="C12" s="234" t="n"/>
@@ -2714,7 +2714,7 @@
       <c r="AX12" s="234" t="n"/>
       <c r="AY12" s="234" t="n"/>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="58.5" customHeight="1">
       <c r="A13" s="234" t="n"/>
       <c r="B13" s="234" t="n"/>
       <c r="C13" s="234" t="n"/>
@@ -2767,7 +2767,7 @@
       <c r="AX13" s="234" t="n"/>
       <c r="AY13" s="234" t="n"/>
     </row>
-    <row r="14" ht="18" customHeight="1">
+    <row r="14" ht="58.5" customHeight="1">
       <c r="A14" s="234" t="n"/>
       <c r="B14" s="234" t="n"/>
       <c r="C14" s="234" t="n"/>
@@ -2820,7 +2820,7 @@
       <c r="AX14" s="234" t="n"/>
       <c r="AY14" s="234" t="n"/>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15" ht="58.5" customHeight="1">
       <c r="A15" s="234" t="n"/>
       <c r="B15" s="234" t="n"/>
       <c r="C15" s="234" t="n"/>
@@ -2873,7 +2873,7 @@
       <c r="AX15" s="234" t="n"/>
       <c r="AY15" s="234" t="n"/>
     </row>
-    <row r="16" ht="18" customHeight="1">
+    <row r="16" ht="58.5" customHeight="1">
       <c r="A16" s="234" t="n"/>
       <c r="B16" s="234" t="n"/>
       <c r="C16" s="234" t="n"/>
@@ -2926,7 +2926,7 @@
       <c r="AX16" s="234" t="n"/>
       <c r="AY16" s="234" t="n"/>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="58.5" customHeight="1">
       <c r="A17" s="234" t="n"/>
       <c r="B17" s="234" t="n"/>
       <c r="C17" s="234" t="n"/>
@@ -2979,7 +2979,7 @@
       <c r="AX17" s="234" t="n"/>
       <c r="AY17" s="234" t="n"/>
     </row>
-    <row r="18" ht="18" customHeight="1">
+    <row r="18" ht="58.5" customHeight="1">
       <c r="A18" s="234" t="n"/>
       <c r="B18" s="234" t="n"/>
       <c r="C18" s="234" t="n"/>
@@ -3032,7 +3032,7 @@
       <c r="AX18" s="234" t="n"/>
       <c r="AY18" s="234" t="n"/>
     </row>
-    <row r="19" ht="18" customHeight="1">
+    <row r="19" ht="58.5" customHeight="1">
       <c r="A19" s="234" t="n"/>
       <c r="B19" s="234" t="n"/>
       <c r="C19" s="234" t="n"/>
@@ -3085,7 +3085,7 @@
       <c r="AX19" s="234" t="n"/>
       <c r="AY19" s="234" t="n"/>
     </row>
-    <row r="20" ht="18" customHeight="1">
+    <row r="20" ht="58.5" customHeight="1">
       <c r="A20" s="234" t="n"/>
       <c r="B20" s="234" t="n"/>
       <c r="C20" s="234" t="n"/>
@@ -3138,7 +3138,7 @@
       <c r="AX20" s="234" t="n"/>
       <c r="AY20" s="234" t="n"/>
     </row>
-    <row r="21" ht="18" customHeight="1">
+    <row r="21" ht="58.5" customHeight="1">
       <c r="A21" s="234" t="n"/>
       <c r="B21" s="234" t="n"/>
       <c r="C21" s="234" t="n"/>
@@ -3191,7 +3191,7 @@
       <c r="AX21" s="234" t="n"/>
       <c r="AY21" s="234" t="n"/>
     </row>
-    <row r="22" ht="18" customHeight="1">
+    <row r="22" ht="49.5" customHeight="1">
       <c r="A22" s="234" t="n"/>
       <c r="B22" s="234" t="n"/>
       <c r="C22" s="234" t="n"/>
@@ -3244,7 +3244,7 @@
       <c r="AX22" s="234" t="n"/>
       <c r="AY22" s="234" t="n"/>
     </row>
-    <row r="23" ht="18" customHeight="1">
+    <row r="23" ht="49.5" customHeight="1">
       <c r="A23" s="234" t="n"/>
       <c r="B23" s="234" t="n"/>
       <c r="C23" s="234" t="n"/>
@@ -3297,7 +3297,7 @@
       <c r="AX23" s="234" t="n"/>
       <c r="AY23" s="234" t="n"/>
     </row>
-    <row r="24" ht="18" customHeight="1">
+    <row r="24" ht="49.5" customHeight="1">
       <c r="A24" s="234" t="n"/>
       <c r="B24" s="234" t="n"/>
       <c r="C24" s="234" t="n"/>
@@ -3350,7 +3350,7 @@
       <c r="AX24" s="234" t="n"/>
       <c r="AY24" s="234" t="n"/>
     </row>
-    <row r="25" ht="18" customHeight="1">
+    <row r="25" ht="49.5" customHeight="1">
       <c r="A25" s="234" t="n"/>
       <c r="B25" s="234" t="n"/>
       <c r="C25" s="234" t="n"/>
@@ -3403,7 +3403,7 @@
       <c r="AX25" s="234" t="n"/>
       <c r="AY25" s="234" t="n"/>
     </row>
-    <row r="26" ht="18" customHeight="1">
+    <row r="26" ht="49.5" customHeight="1">
       <c r="A26" s="234" t="n"/>
       <c r="B26" s="234" t="n"/>
       <c r="C26" s="234" t="n"/>
@@ -3456,7 +3456,7 @@
       <c r="AX26" s="234" t="n"/>
       <c r="AY26" s="234" t="n"/>
     </row>
-    <row r="27" ht="18" customHeight="1">
+    <row r="27" ht="49.5" customHeight="1">
       <c r="A27" s="234" t="n"/>
       <c r="B27" s="234" t="n"/>
       <c r="C27" s="234" t="n"/>
@@ -3509,7 +3509,7 @@
       <c r="AX27" s="234" t="n"/>
       <c r="AY27" s="234" t="n"/>
     </row>
-    <row r="28" ht="18" customHeight="1">
+    <row r="28" ht="49.5" customHeight="1">
       <c r="A28" s="234" t="n"/>
       <c r="B28" s="234" t="n"/>
       <c r="C28" s="234" t="n"/>
@@ -3562,7 +3562,7 @@
       <c r="AX28" s="234" t="n"/>
       <c r="AY28" s="234" t="n"/>
     </row>
-    <row r="29" ht="18" customHeight="1">
+    <row r="29" ht="51" customHeight="1">
       <c r="A29" s="234" t="n"/>
       <c r="B29" s="234" t="n"/>
       <c r="C29" s="234" t="n"/>
@@ -3615,7 +3615,7 @@
       <c r="AX29" s="234" t="n"/>
       <c r="AY29" s="234" t="n"/>
     </row>
-    <row r="30" ht="18" customHeight="1" thickBot="1">
+    <row r="30" ht="51" customHeight="1" thickBot="1">
       <c r="A30" s="234" t="n"/>
       <c r="B30" s="234" t="n"/>
       <c r="C30" s="234" t="n"/>
@@ -3668,7 +3668,7 @@
       <c r="AX30" s="234" t="n"/>
       <c r="AY30" s="234" t="n"/>
     </row>
-    <row r="31" ht="18" customHeight="1" thickBot="1">
+    <row r="31" ht="51" customHeight="1" thickBot="1">
       <c r="A31" s="234" t="n"/>
       <c r="B31" s="234" t="n"/>
       <c r="C31" s="234" t="n"/>
@@ -3721,7 +3721,7 @@
       <c r="AX31" s="234" t="n"/>
       <c r="AY31" s="234" t="n"/>
     </row>
-    <row r="32" ht="18" customHeight="1">
+    <row r="32" ht="51" customHeight="1">
       <c r="A32" s="234" t="n"/>
       <c r="B32" s="234" t="n"/>
       <c r="C32" s="234" t="n"/>
@@ -3774,7 +3774,7 @@
       <c r="AX32" s="234" t="n"/>
       <c r="AY32" s="234" t="n"/>
     </row>
-    <row r="33" ht="18" customHeight="1">
+    <row r="33" ht="51" customHeight="1">
       <c r="A33" s="234" t="n"/>
       <c r="B33" s="234" t="n"/>
       <c r="C33" s="234" t="n"/>
@@ -3827,7 +3827,7 @@
       <c r="AX33" s="234" t="n"/>
       <c r="AY33" s="234" t="n"/>
     </row>
-    <row r="34" ht="18" customHeight="1" thickBot="1">
+    <row r="34" ht="51" customHeight="1" thickBot="1">
       <c r="A34" s="234" t="n"/>
       <c r="B34" s="234" t="n"/>
       <c r="C34" s="234" t="n"/>
@@ -3880,7 +3880,7 @@
       <c r="AX34" s="234" t="n"/>
       <c r="AY34" s="234" t="n"/>
     </row>
-    <row r="35" ht="18" customHeight="1">
+    <row r="35" ht="51" customHeight="1">
       <c r="A35" s="234" t="n"/>
       <c r="B35" s="234" t="n"/>
       <c r="C35" s="234" t="n"/>
@@ -3933,7 +3933,7 @@
       <c r="AX35" s="234" t="n"/>
       <c r="AY35" s="234" t="n"/>
     </row>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="51" customHeight="1">
       <c r="A36" s="234" t="n"/>
       <c r="B36" s="234" t="n"/>
       <c r="C36" s="234" t="n"/>
@@ -3986,7 +3986,7 @@
       <c r="AX36" s="234" t="n"/>
       <c r="AY36" s="234" t="n"/>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="51" customHeight="1">
       <c r="A37" s="234" t="n"/>
       <c r="B37" s="234" t="n"/>
       <c r="C37" s="234" t="n"/>
@@ -4039,7 +4039,7 @@
       <c r="AX37" s="234" t="n"/>
       <c r="AY37" s="234" t="n"/>
     </row>
-    <row r="38" ht="18" customHeight="1">
+    <row r="38" ht="51" customHeight="1">
       <c r="A38" s="234" t="n"/>
       <c r="B38" s="234" t="n"/>
       <c r="C38" s="234" t="n"/>
@@ -4092,7 +4092,7 @@
       <c r="AX38" s="234" t="n"/>
       <c r="AY38" s="234" t="n"/>
     </row>
-    <row r="39" ht="18" customHeight="1">
+    <row r="39" ht="51" customHeight="1">
       <c r="A39" s="234" t="n"/>
       <c r="B39" s="234" t="n"/>
       <c r="C39" s="234" t="n"/>
@@ -4145,7 +4145,7 @@
       <c r="AX39" s="234" t="n"/>
       <c r="AY39" s="234" t="n"/>
     </row>
-    <row r="40" ht="18" customHeight="1" thickBot="1">
+    <row r="40" ht="51" customHeight="1" thickBot="1">
       <c r="A40" s="234" t="n"/>
       <c r="B40" s="234" t="n"/>
       <c r="C40" s="234" t="n"/>
@@ -4240,7 +4240,7 @@
     <mergeCell ref="H10:H11"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup orientation="landscape" paperSize="5" scale="39"/>
+  <pageSetup orientation="landscape" paperSize="5" fitToHeight="1" fitToWidth="1"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="37" min="1" max="40" man="1"/>
   </colBreaks>

</xml_diff>